<commit_message>
initial density matrix guess
</commit_message>
<xml_diff>
--- a/hamiltonian_core_matrix.xlsx
+++ b/hamiltonian_core_matrix.xlsx
@@ -418,16 +418,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>-2808.419024807049</v>
+        <v>4.139159679920277</v>
       </c>
       <c r="B1" t="n">
-        <v>0</v>
+        <v>4.439872370214957</v>
       </c>
       <c r="C1" t="n">
-        <v>0</v>
+        <v>2.301202142182699</v>
       </c>
       <c r="D1" t="n">
-        <v>0</v>
+        <v>2.272781618054275</v>
       </c>
       <c r="E1" t="n">
         <v>0</v>
@@ -436,7 +436,7 @@
         <v>0</v>
       </c>
       <c r="G1" t="n">
-        <v>0</v>
+        <v>0.03612803534483141</v>
       </c>
       <c r="H1" t="n">
         <v>0</v>
@@ -445,7 +445,7 @@
         <v>0</v>
       </c>
       <c r="J1" t="n">
-        <v>0</v>
+        <v>0.03074431601516749</v>
       </c>
       <c r="K1" t="n">
         <v>0</v>
@@ -454,19 +454,19 @@
         <v>0</v>
       </c>
       <c r="M1" t="n">
-        <v>0</v>
+        <v>0.03310305217715067</v>
       </c>
       <c r="N1" t="n">
-        <v>0</v>
+        <v>-1.164331493840184e-07</v>
       </c>
       <c r="O1" t="n">
-        <v>0</v>
+        <v>0.00908727878601103</v>
       </c>
       <c r="P1" t="n">
-        <v>0</v>
+        <v>0.5454495722126946</v>
       </c>
       <c r="Q1" t="n">
-        <v>0</v>
+        <v>1.449521828263224</v>
       </c>
       <c r="R1" t="n">
         <v>0</v>
@@ -475,7 +475,7 @@
         <v>0</v>
       </c>
       <c r="T1" t="n">
-        <v>0</v>
+        <v>-0.004917756917705785</v>
       </c>
       <c r="U1" t="n">
         <v>0</v>
@@ -484,7 +484,7 @@
         <v>0</v>
       </c>
       <c r="W1" t="n">
-        <v>0</v>
+        <v>-0.4570860794626933</v>
       </c>
       <c r="X1" t="n">
         <v>0</v>
@@ -493,19 +493,19 @@
         <v>0</v>
       </c>
       <c r="Z1" t="n">
-        <v>0</v>
+        <v>-1.16868944234641</v>
       </c>
       <c r="AA1" t="n">
-        <v>0</v>
+        <v>0.05955589180169553</v>
       </c>
       <c r="AB1" t="n">
-        <v>0</v>
+        <v>1.418553104775894</v>
       </c>
       <c r="AC1" t="n">
-        <v>0</v>
+        <v>1.831416724125386</v>
       </c>
       <c r="AD1" t="n">
-        <v>0</v>
+        <v>2.138875613550525</v>
       </c>
       <c r="AE1" t="n">
         <v>0</v>
@@ -514,7 +514,7 @@
         <v>0</v>
       </c>
       <c r="AG1" t="n">
-        <v>0</v>
+        <v>-0.5964506393073215</v>
       </c>
       <c r="AH1" t="n">
         <v>0</v>
@@ -523,7 +523,7 @@
         <v>0</v>
       </c>
       <c r="AJ1" t="n">
-        <v>0</v>
+        <v>-0.773537103112676</v>
       </c>
       <c r="AK1" t="n">
         <v>0</v>
@@ -532,21 +532,21 @@
         <v>0</v>
       </c>
       <c r="AM1" t="n">
-        <v>0</v>
+        <v>-0.8272631971284673</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0</v>
+        <v>4.439872370214957</v>
       </c>
       <c r="B2" t="n">
-        <v>-2808.419024807045</v>
+        <v>16.42792488608161</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>15.60550082657199</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>16.46798512610517</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -555,7 +555,7 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>0.5819261365744327</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -564,7 +564,7 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>1.475462685247075</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -573,19 +573,19 @@
         <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>2.723285606951114</v>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
+        <v>0.00908727878601104</v>
       </c>
       <c r="O2" t="n">
-        <v>0</v>
+        <v>0.3020651239926924</v>
       </c>
       <c r="P2" t="n">
-        <v>0</v>
+        <v>5.049791993425586</v>
       </c>
       <c r="Q2" t="n">
-        <v>0</v>
+        <v>11.17828061640937</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -594,7 +594,7 @@
         <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>0</v>
+        <v>-0.1787429074991289</v>
       </c>
       <c r="U2" t="n">
         <v>0</v>
@@ -603,7 +603,7 @@
         <v>0</v>
       </c>
       <c r="W2" t="n">
-        <v>0</v>
+        <v>-3.971360158404172</v>
       </c>
       <c r="X2" t="n">
         <v>0</v>
@@ -612,19 +612,19 @@
         <v>0</v>
       </c>
       <c r="Z2" t="n">
-        <v>0</v>
+        <v>-9.21881277318213</v>
       </c>
       <c r="AA2" t="n">
-        <v>0</v>
+        <v>1.576222444784207</v>
       </c>
       <c r="AB2" t="n">
-        <v>0</v>
+        <v>11.44831120197395</v>
       </c>
       <c r="AC2" t="n">
-        <v>0</v>
+        <v>13.67190820985699</v>
       </c>
       <c r="AD2" t="n">
-        <v>0</v>
+        <v>15.84842555965021</v>
       </c>
       <c r="AE2" t="n">
         <v>0</v>
@@ -633,7 +633,7 @@
         <v>0</v>
       </c>
       <c r="AG2" t="n">
-        <v>0</v>
+        <v>-3.602246001538805</v>
       </c>
       <c r="AH2" t="n">
         <v>0</v>
@@ -642,7 +642,7 @@
         <v>0</v>
       </c>
       <c r="AJ2" t="n">
-        <v>0</v>
+        <v>-5.530407213910946</v>
       </c>
       <c r="AK2" t="n">
         <v>0</v>
@@ -651,21 +651,21 @@
         <v>0</v>
       </c>
       <c r="AM2" t="n">
-        <v>0</v>
+        <v>-5.139031126558099</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0</v>
+        <v>2.301202142182699</v>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>15.60550082657199</v>
       </c>
       <c r="C3" t="n">
-        <v>-2774.528233268392</v>
+        <v>25.36028734692464</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>51.91216676124913</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -674,7 +674,7 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>1.475462685247074</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -683,7 +683,7 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>6.912828115024684</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -692,19 +692,19 @@
         <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>13.76609940898933</v>
       </c>
       <c r="N3" t="n">
-        <v>0</v>
+        <v>0.5454495722126947</v>
       </c>
       <c r="O3" t="n">
-        <v>0</v>
+        <v>5.049791993425586</v>
       </c>
       <c r="P3" t="n">
-        <v>0</v>
+        <v>18.74092126346848</v>
       </c>
       <c r="Q3" t="n">
-        <v>0</v>
+        <v>38.39856510910838</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -713,7 +713,7 @@
         <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>0</v>
+        <v>-1.124625794116042</v>
       </c>
       <c r="U3" t="n">
         <v>0</v>
@@ -722,7 +722,7 @@
         <v>0</v>
       </c>
       <c r="W3" t="n">
-        <v>0</v>
+        <v>-10.15530698853429</v>
       </c>
       <c r="X3" t="n">
         <v>0</v>
@@ -731,19 +731,19 @@
         <v>0</v>
       </c>
       <c r="Z3" t="n">
-        <v>0</v>
+        <v>-23.69877968611681</v>
       </c>
       <c r="AA3" t="n">
-        <v>0</v>
+        <v>3.508714021200267</v>
       </c>
       <c r="AB3" t="n">
-        <v>0</v>
+        <v>24.12121622154257</v>
       </c>
       <c r="AC3" t="n">
-        <v>0</v>
+        <v>38.5077583072274</v>
       </c>
       <c r="AD3" t="n">
-        <v>0</v>
+        <v>55.30620345657083</v>
       </c>
       <c r="AE3" t="n">
         <v>0</v>
@@ -752,7 +752,7 @@
         <v>0</v>
       </c>
       <c r="AG3" t="n">
-        <v>0</v>
+        <v>-3.031657194942603</v>
       </c>
       <c r="AH3" t="n">
         <v>0</v>
@@ -761,7 +761,7 @@
         <v>0</v>
       </c>
       <c r="AJ3" t="n">
-        <v>0</v>
+        <v>-7.76217934737705</v>
       </c>
       <c r="AK3" t="n">
         <v>0</v>
@@ -770,21 +770,21 @@
         <v>0</v>
       </c>
       <c r="AM3" t="n">
-        <v>0</v>
+        <v>-6.456376566773256</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0</v>
+        <v>2.272781618054275</v>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>16.46798512610517</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>51.91216676124913</v>
       </c>
       <c r="D4" t="n">
-        <v>-555.030887280054</v>
+        <v>39.05462463097899</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -793,7 +793,7 @@
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>2.723285606951114</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -802,7 +802,7 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>13.76609940898933</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -811,19 +811,19 @@
         <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>43.12718909070011</v>
       </c>
       <c r="N4" t="n">
-        <v>0</v>
+        <v>1.449521828263224</v>
       </c>
       <c r="O4" t="n">
-        <v>0</v>
+        <v>11.17828061640937</v>
       </c>
       <c r="P4" t="n">
-        <v>0</v>
+        <v>38.39856510910838</v>
       </c>
       <c r="Q4" t="n">
-        <v>0</v>
+        <v>95.71472975852407</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -832,7 +832,7 @@
         <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>0</v>
+        <v>-2.088945385966567</v>
       </c>
       <c r="U4" t="n">
         <v>0</v>
@@ -841,7 +841,7 @@
         <v>0</v>
       </c>
       <c r="W4" t="n">
-        <v>0</v>
+        <v>-17.40650157142676</v>
       </c>
       <c r="X4" t="n">
         <v>0</v>
@@ -850,19 +850,19 @@
         <v>0</v>
       </c>
       <c r="Z4" t="n">
-        <v>0</v>
+        <v>-47.39092645945157</v>
       </c>
       <c r="AA4" t="n">
-        <v>0</v>
+        <v>4.512122142873354</v>
       </c>
       <c r="AB4" t="n">
-        <v>0</v>
+        <v>36.21567214747493</v>
       </c>
       <c r="AC4" t="n">
-        <v>0</v>
+        <v>78.68980267650088</v>
       </c>
       <c r="AD4" t="n">
-        <v>0</v>
+        <v>151.1499475879253</v>
       </c>
       <c r="AE4" t="n">
         <v>0</v>
@@ -871,7 +871,7 @@
         <v>0</v>
       </c>
       <c r="AG4" t="n">
-        <v>0</v>
+        <v>-0.5487270400261994</v>
       </c>
       <c r="AH4" t="n">
         <v>0</v>
@@ -880,7 +880,7 @@
         <v>0</v>
       </c>
       <c r="AJ4" t="n">
-        <v>0</v>
+        <v>-3.978407090882079</v>
       </c>
       <c r="AK4" t="n">
         <v>0</v>
@@ -889,7 +889,7 @@
         <v>0</v>
       </c>
       <c r="AM4" t="n">
-        <v>0</v>
+        <v>-11.56233920550879</v>
       </c>
     </row>
     <row r="5">
@@ -906,7 +906,7 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>-555.0308872800529</v>
+        <v>1.192134315798659</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -915,7 +915,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>1.766832501424194</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -924,7 +924,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>1.382854560945209</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
@@ -945,7 +945,7 @@
         <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>0</v>
+        <v>0.01064078252761629</v>
       </c>
       <c r="S5" t="n">
         <v>0</v>
@@ -954,7 +954,7 @@
         <v>0</v>
       </c>
       <c r="U5" t="n">
-        <v>0</v>
+        <v>0.3758371805596659</v>
       </c>
       <c r="V5" t="n">
         <v>0</v>
@@ -963,7 +963,7 @@
         <v>0</v>
       </c>
       <c r="X5" t="n">
-        <v>0</v>
+        <v>0.8333571581880173</v>
       </c>
       <c r="Y5" t="n">
         <v>0</v>
@@ -984,7 +984,7 @@
         <v>0</v>
       </c>
       <c r="AE5" t="n">
-        <v>0</v>
+        <v>0.7651230248262965</v>
       </c>
       <c r="AF5" t="n">
         <v>0</v>
@@ -993,7 +993,7 @@
         <v>0</v>
       </c>
       <c r="AH5" t="n">
-        <v>0</v>
+        <v>1.27280487236772</v>
       </c>
       <c r="AI5" t="n">
         <v>0</v>
@@ -1002,7 +1002,7 @@
         <v>0</v>
       </c>
       <c r="AK5" t="n">
-        <v>0</v>
+        <v>1.097514897426634</v>
       </c>
       <c r="AL5" t="n">
         <v>0</v>
@@ -1028,7 +1028,7 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>-485.6056516142546</v>
+        <v>1.192134315798659</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -1037,7 +1037,7 @@
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>1.766832501424194</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -1046,7 +1046,7 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>0</v>
+        <v>1.382854560945209</v>
       </c>
       <c r="M6" t="n">
         <v>0</v>
@@ -1067,7 +1067,7 @@
         <v>0</v>
       </c>
       <c r="S6" t="n">
-        <v>0</v>
+        <v>0.01064078252761629</v>
       </c>
       <c r="T6" t="n">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         <v>0</v>
       </c>
       <c r="V6" t="n">
-        <v>0</v>
+        <v>0.3758371805596659</v>
       </c>
       <c r="W6" t="n">
         <v>0</v>
@@ -1085,7 +1085,7 @@
         <v>0</v>
       </c>
       <c r="Y6" t="n">
-        <v>0</v>
+        <v>0.8333571581880168</v>
       </c>
       <c r="Z6" t="n">
         <v>0</v>
@@ -1106,7 +1106,7 @@
         <v>0</v>
       </c>
       <c r="AF6" t="n">
-        <v>0</v>
+        <v>0.7651230248262962</v>
       </c>
       <c r="AG6" t="n">
         <v>0</v>
@@ -1115,7 +1115,7 @@
         <v>0</v>
       </c>
       <c r="AI6" t="n">
-        <v>0</v>
+        <v>1.272804872367719</v>
       </c>
       <c r="AJ6" t="n">
         <v>0</v>
@@ -1124,7 +1124,7 @@
         <v>0</v>
       </c>
       <c r="AL6" t="n">
-        <v>0</v>
+        <v>1.097514897426633</v>
       </c>
       <c r="AM6" t="n">
         <v>0</v>
@@ -1132,16 +1132,16 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0</v>
+        <v>0.03612803534483141</v>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>0.5819261365744327</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>1.475462685247074</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>2.723285606951114</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -1150,7 +1150,7 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>-416.2016062272453</v>
+        <v>1.477838631755247</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -1159,7 +1159,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>3.250101211246582</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -1168,19 +1168,19 @@
         <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>3.194957394976628</v>
       </c>
       <c r="N7" t="n">
-        <v>0</v>
+        <v>0.004917756917705804</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>0.178742907499129</v>
       </c>
       <c r="P7" t="n">
-        <v>0</v>
+        <v>1.124625794116042</v>
       </c>
       <c r="Q7" t="n">
-        <v>0</v>
+        <v>2.088945385966567</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -1189,7 +1189,7 @@
         <v>0</v>
       </c>
       <c r="T7" t="n">
-        <v>0</v>
+        <v>-0.2169371577703999</v>
       </c>
       <c r="U7" t="n">
         <v>0</v>
@@ -1198,7 +1198,7 @@
         <v>0</v>
       </c>
       <c r="W7" t="n">
-        <v>0</v>
+        <v>-1.248713956425855</v>
       </c>
       <c r="X7" t="n">
         <v>0</v>
@@ -1207,19 +1207,19 @@
         <v>0</v>
       </c>
       <c r="Z7" t="n">
-        <v>0</v>
+        <v>-0.930653878475391</v>
       </c>
       <c r="AA7" t="n">
-        <v>0</v>
+        <v>0.6378678045689179</v>
       </c>
       <c r="AB7" t="n">
-        <v>0</v>
+        <v>2.760336696370763</v>
       </c>
       <c r="AC7" t="n">
-        <v>0</v>
+        <v>2.520531082126993</v>
       </c>
       <c r="AD7" t="n">
-        <v>0</v>
+        <v>2.802640033063934</v>
       </c>
       <c r="AE7" t="n">
         <v>0</v>
@@ -1228,7 +1228,7 @@
         <v>0</v>
       </c>
       <c r="AG7" t="n">
-        <v>0</v>
+        <v>-0.2074482860328148</v>
       </c>
       <c r="AH7" t="n">
         <v>0</v>
@@ -1237,7 +1237,7 @@
         <v>0</v>
       </c>
       <c r="AJ7" t="n">
-        <v>0</v>
+        <v>0.8149003037378533</v>
       </c>
       <c r="AK7" t="n">
         <v>0</v>
@@ -1246,7 +1246,7 @@
         <v>0</v>
       </c>
       <c r="AM7" t="n">
-        <v>0</v>
+        <v>1.178655034612895</v>
       </c>
     </row>
     <row r="8">
@@ -1263,7 +1263,7 @@
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>1.766832501424194</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -1272,7 +1272,7 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>-416.2016062272453</v>
+        <v>-13.40329958962834</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -1281,7 +1281,7 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>20.18728619194507</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -1302,7 +1302,7 @@
         <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>0</v>
+        <v>0.3758371805596656</v>
       </c>
       <c r="S8" t="n">
         <v>0</v>
@@ -1311,7 +1311,7 @@
         <v>0</v>
       </c>
       <c r="U8" t="n">
-        <v>0</v>
+        <v>4.550080082221125</v>
       </c>
       <c r="V8" t="n">
         <v>0</v>
@@ -1320,7 +1320,7 @@
         <v>0</v>
       </c>
       <c r="X8" t="n">
-        <v>0</v>
+        <v>12.8982716519249</v>
       </c>
       <c r="Y8" t="n">
         <v>0</v>
@@ -1341,7 +1341,7 @@
         <v>0</v>
       </c>
       <c r="AE8" t="n">
-        <v>0</v>
+        <v>3.676068662738705</v>
       </c>
       <c r="AF8" t="n">
         <v>0</v>
@@ -1350,7 +1350,7 @@
         <v>0</v>
       </c>
       <c r="AH8" t="n">
-        <v>0</v>
+        <v>13.81389572988589</v>
       </c>
       <c r="AI8" t="n">
         <v>0</v>
@@ -1359,7 +1359,7 @@
         <v>0</v>
       </c>
       <c r="AK8" t="n">
-        <v>0</v>
+        <v>18.37925462552074</v>
       </c>
       <c r="AL8" t="n">
         <v>0</v>
@@ -1385,7 +1385,7 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>1.766832501424194</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -1394,7 +1394,7 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>-412.5316766388101</v>
+        <v>-13.40329958962834</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -1403,7 +1403,7 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>20.18728619194507</v>
       </c>
       <c r="M9" t="n">
         <v>0</v>
@@ -1424,7 +1424,7 @@
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>0</v>
+        <v>0.3758371805596658</v>
       </c>
       <c r="T9" t="n">
         <v>0</v>
@@ -1433,7 +1433,7 @@
         <v>0</v>
       </c>
       <c r="V9" t="n">
-        <v>0</v>
+        <v>4.550080082221125</v>
       </c>
       <c r="W9" t="n">
         <v>0</v>
@@ -1442,7 +1442,7 @@
         <v>0</v>
       </c>
       <c r="Y9" t="n">
-        <v>0</v>
+        <v>12.89827165192491</v>
       </c>
       <c r="Z9" t="n">
         <v>0</v>
@@ -1463,7 +1463,7 @@
         <v>0</v>
       </c>
       <c r="AF9" t="n">
-        <v>0</v>
+        <v>3.676068662738704</v>
       </c>
       <c r="AG9" t="n">
         <v>0</v>
@@ -1472,7 +1472,7 @@
         <v>0</v>
       </c>
       <c r="AI9" t="n">
-        <v>0</v>
+        <v>13.81389572988588</v>
       </c>
       <c r="AJ9" t="n">
         <v>0</v>
@@ -1481,7 +1481,7 @@
         <v>0</v>
       </c>
       <c r="AL9" t="n">
-        <v>0</v>
+        <v>18.37925462552075</v>
       </c>
       <c r="AM9" t="n">
         <v>0</v>
@@ -1489,16 +1489,16 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0</v>
+        <v>0.03074431601516749</v>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>1.475462685247075</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>6.912828115024684</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>13.76609940898933</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -1507,7 +1507,7 @@
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>3.250101211246582</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
@@ -1516,7 +1516,7 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>-156.5590962155348</v>
+        <v>-7.381924980802701</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
@@ -1525,19 +1525,19 @@
         <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>0</v>
+        <v>44.03641252598699</v>
       </c>
       <c r="N10" t="n">
-        <v>0</v>
+        <v>0.4570860794626934</v>
       </c>
       <c r="O10" t="n">
-        <v>0</v>
+        <v>3.971360158404171</v>
       </c>
       <c r="P10" t="n">
-        <v>0</v>
+        <v>10.15530698853429</v>
       </c>
       <c r="Q10" t="n">
-        <v>0</v>
+        <v>17.40650157142676</v>
       </c>
       <c r="R10" t="n">
         <v>0</v>
@@ -1546,7 +1546,7 @@
         <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>0</v>
+        <v>-1.248713956425854</v>
       </c>
       <c r="U10" t="n">
         <v>0</v>
@@ -1555,7 +1555,7 @@
         <v>0</v>
       </c>
       <c r="W10" t="n">
-        <v>0</v>
+        <v>-5.357830832620333</v>
       </c>
       <c r="X10" t="n">
         <v>0</v>
@@ -1564,19 +1564,19 @@
         <v>0</v>
       </c>
       <c r="Z10" t="n">
-        <v>0</v>
+        <v>0.3636216678918136</v>
       </c>
       <c r="AA10" t="n">
-        <v>0</v>
+        <v>1.586326549568464</v>
       </c>
       <c r="AB10" t="n">
-        <v>0</v>
+        <v>10.86627905110093</v>
       </c>
       <c r="AC10" t="n">
-        <v>0</v>
+        <v>15.44425040665211</v>
       </c>
       <c r="AD10" t="n">
-        <v>0</v>
+        <v>23.12502089407928</v>
       </c>
       <c r="AE10" t="n">
         <v>0</v>
@@ -1585,7 +1585,7 @@
         <v>0</v>
       </c>
       <c r="AG10" t="n">
-        <v>0</v>
+        <v>4.911791365184697</v>
       </c>
       <c r="AH10" t="n">
         <v>0</v>
@@ -1594,7 +1594,7 @@
         <v>0</v>
       </c>
       <c r="AJ10" t="n">
-        <v>0</v>
+        <v>16.06636222813914</v>
       </c>
       <c r="AK10" t="n">
         <v>0</v>
@@ -1603,7 +1603,7 @@
         <v>0</v>
       </c>
       <c r="AM10" t="n">
-        <v>0</v>
+        <v>28.31024971547307</v>
       </c>
     </row>
     <row r="11">
@@ -1620,7 +1620,7 @@
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>1.382854560945209</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
@@ -1629,7 +1629,7 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>20.18728619194507</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -1638,7 +1638,7 @@
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>-66.82533526852976</v>
+        <v>-486.8332616027242</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -1659,7 +1659,7 @@
         <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>0</v>
+        <v>0.8333571581880166</v>
       </c>
       <c r="S11" t="n">
         <v>0</v>
@@ -1668,7 +1668,7 @@
         <v>0</v>
       </c>
       <c r="U11" t="n">
-        <v>0</v>
+        <v>12.8982716519249</v>
       </c>
       <c r="V11" t="n">
         <v>0</v>
@@ -1677,7 +1677,7 @@
         <v>0</v>
       </c>
       <c r="X11" t="n">
-        <v>0</v>
+        <v>68.09819569804129</v>
       </c>
       <c r="Y11" t="n">
         <v>0</v>
@@ -1698,7 +1698,7 @@
         <v>0</v>
       </c>
       <c r="AE11" t="n">
-        <v>0</v>
+        <v>4.518849650494094</v>
       </c>
       <c r="AF11" t="n">
         <v>0</v>
@@ -1707,7 +1707,7 @@
         <v>0</v>
       </c>
       <c r="AH11" t="n">
-        <v>0</v>
+        <v>37.24777675403165</v>
       </c>
       <c r="AI11" t="n">
         <v>0</v>
@@ -1716,7 +1716,7 @@
         <v>0</v>
       </c>
       <c r="AK11" t="n">
-        <v>0</v>
+        <v>129.7348004269145</v>
       </c>
       <c r="AL11" t="n">
         <v>0</v>
@@ -1742,7 +1742,7 @@
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>1.382854560945209</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -1751,7 +1751,7 @@
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>20.18728619194507</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -1760,7 +1760,7 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>-66.82533526852974</v>
+        <v>-486.8332616027242</v>
       </c>
       <c r="M12" t="n">
         <v>0</v>
@@ -1781,7 +1781,7 @@
         <v>0</v>
       </c>
       <c r="S12" t="n">
-        <v>0</v>
+        <v>0.8333571581880166</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1790,7 +1790,7 @@
         <v>0</v>
       </c>
       <c r="V12" t="n">
-        <v>0</v>
+        <v>12.8982716519249</v>
       </c>
       <c r="W12" t="n">
         <v>0</v>
@@ -1799,7 +1799,7 @@
         <v>0</v>
       </c>
       <c r="Y12" t="n">
-        <v>0</v>
+        <v>68.09819569804129</v>
       </c>
       <c r="Z12" t="n">
         <v>0</v>
@@ -1820,7 +1820,7 @@
         <v>0</v>
       </c>
       <c r="AF12" t="n">
-        <v>0</v>
+        <v>4.518849650494094</v>
       </c>
       <c r="AG12" t="n">
         <v>0</v>
@@ -1829,7 +1829,7 @@
         <v>0</v>
       </c>
       <c r="AI12" t="n">
-        <v>0</v>
+        <v>37.24777675403165</v>
       </c>
       <c r="AJ12" t="n">
         <v>0</v>
@@ -1838,7 +1838,7 @@
         <v>0</v>
       </c>
       <c r="AL12" t="n">
-        <v>0</v>
+        <v>129.7348004269146</v>
       </c>
       <c r="AM12" t="n">
         <v>0</v>
@@ -1846,16 +1846,16 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0</v>
+        <v>0.03310305217715067</v>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>2.723285606951114</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>13.76609940898933</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>43.12718909070011</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
@@ -1864,7 +1864,7 @@
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>3.194957394976628</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -1873,7 +1873,7 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>44.03641252598699</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -1882,19 +1882,19 @@
         <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>-64.09054076946363</v>
+        <v>-436.8057222575121</v>
       </c>
       <c r="N13" t="n">
-        <v>0</v>
+        <v>1.16868944234641</v>
       </c>
       <c r="O13" t="n">
-        <v>0</v>
+        <v>9.218812773182133</v>
       </c>
       <c r="P13" t="n">
-        <v>0</v>
+        <v>23.69877968611682</v>
       </c>
       <c r="Q13" t="n">
-        <v>0</v>
+        <v>47.39092645945158</v>
       </c>
       <c r="R13" t="n">
         <v>0</v>
@@ -1903,7 +1903,7 @@
         <v>0</v>
       </c>
       <c r="T13" t="n">
-        <v>0</v>
+        <v>-0.9306538784753915</v>
       </c>
       <c r="U13" t="n">
         <v>0</v>
@@ -1912,7 +1912,7 @@
         <v>0</v>
       </c>
       <c r="W13" t="n">
-        <v>0</v>
+        <v>0.3636216678918154</v>
       </c>
       <c r="X13" t="n">
         <v>0</v>
@@ -1921,19 +1921,19 @@
         <v>0</v>
       </c>
       <c r="Z13" t="n">
-        <v>0</v>
+        <v>23.68879886756204</v>
       </c>
       <c r="AA13" t="n">
-        <v>0</v>
+        <v>1.877188462822925</v>
       </c>
       <c r="AB13" t="n">
-        <v>0</v>
+        <v>17.2616970864677</v>
       </c>
       <c r="AC13" t="n">
-        <v>0</v>
+        <v>34.62715650309303</v>
       </c>
       <c r="AD13" t="n">
-        <v>0</v>
+        <v>60.6386162974352</v>
       </c>
       <c r="AE13" t="n">
         <v>0</v>
@@ -1942,7 +1942,7 @@
         <v>0</v>
       </c>
       <c r="AG13" t="n">
-        <v>0</v>
+        <v>8.709720073795213</v>
       </c>
       <c r="AH13" t="n">
         <v>0</v>
@@ -1951,7 +1951,7 @@
         <v>0</v>
       </c>
       <c r="AJ13" t="n">
-        <v>0</v>
+        <v>42.56472805406715</v>
       </c>
       <c r="AK13" t="n">
         <v>0</v>
@@ -1960,21 +1960,21 @@
         <v>0</v>
       </c>
       <c r="AM13" t="n">
-        <v>0</v>
+        <v>145.0244454550882</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0</v>
+        <v>-1.164331493840184e-07</v>
       </c>
       <c r="B14" t="n">
-        <v>0</v>
+        <v>0.00908727878601104</v>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>0.5454495722126947</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1.449521828263224</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
@@ -1983,7 +1983,7 @@
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>0.004917756917705804</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -1992,7 +1992,7 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>0.4570860794626934</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
@@ -2001,19 +2001,19 @@
         <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>0</v>
+        <v>1.16868944234641</v>
       </c>
       <c r="N14" t="n">
-        <v>-59.02535540349962</v>
+        <v>4.139159679920277</v>
       </c>
       <c r="O14" t="n">
-        <v>0</v>
+        <v>4.439872370214957</v>
       </c>
       <c r="P14" t="n">
-        <v>0</v>
+        <v>2.301202142182699</v>
       </c>
       <c r="Q14" t="n">
-        <v>0</v>
+        <v>2.272781618054275</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
@@ -2022,7 +2022,7 @@
         <v>0</v>
       </c>
       <c r="T14" t="n">
-        <v>0</v>
+        <v>-0.03612803534483141</v>
       </c>
       <c r="U14" t="n">
         <v>0</v>
@@ -2031,7 +2031,7 @@
         <v>0</v>
       </c>
       <c r="W14" t="n">
-        <v>0</v>
+        <v>-0.03074431601516749</v>
       </c>
       <c r="X14" t="n">
         <v>0</v>
@@ -2040,19 +2040,19 @@
         <v>0</v>
       </c>
       <c r="Z14" t="n">
-        <v>0</v>
+        <v>-0.03310305217715067</v>
       </c>
       <c r="AA14" t="n">
-        <v>0</v>
+        <v>0.05955589180169553</v>
       </c>
       <c r="AB14" t="n">
-        <v>0</v>
+        <v>1.418553104775894</v>
       </c>
       <c r="AC14" t="n">
-        <v>0</v>
+        <v>1.831416724125386</v>
       </c>
       <c r="AD14" t="n">
-        <v>0</v>
+        <v>2.138875613550525</v>
       </c>
       <c r="AE14" t="n">
         <v>0</v>
@@ -2061,7 +2061,7 @@
         <v>0</v>
       </c>
       <c r="AG14" t="n">
-        <v>0</v>
+        <v>0.5964506393073215</v>
       </c>
       <c r="AH14" t="n">
         <v>0</v>
@@ -2070,7 +2070,7 @@
         <v>0</v>
       </c>
       <c r="AJ14" t="n">
-        <v>0</v>
+        <v>0.773537103112676</v>
       </c>
       <c r="AK14" t="n">
         <v>0</v>
@@ -2079,21 +2079,21 @@
         <v>0</v>
       </c>
       <c r="AM14" t="n">
-        <v>0</v>
+        <v>0.8272631971284673</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0</v>
+        <v>0.00908727878601103</v>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>0.3020651239926924</v>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>5.049791993425586</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>11.17828061640937</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -2102,7 +2102,7 @@
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>0.178742907499129</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -2111,7 +2111,7 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>3.971360158404171</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -2120,19 +2120,19 @@
         <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>9.218812773182133</v>
       </c>
       <c r="N15" t="n">
-        <v>0</v>
+        <v>4.439872370214957</v>
       </c>
       <c r="O15" t="n">
-        <v>-28.16159727442432</v>
+        <v>16.42792488608161</v>
       </c>
       <c r="P15" t="n">
-        <v>0</v>
+        <v>15.60550082657199</v>
       </c>
       <c r="Q15" t="n">
-        <v>0</v>
+        <v>16.46798512610517</v>
       </c>
       <c r="R15" t="n">
         <v>0</v>
@@ -2141,7 +2141,7 @@
         <v>0</v>
       </c>
       <c r="T15" t="n">
-        <v>0</v>
+        <v>-0.5819261365744327</v>
       </c>
       <c r="U15" t="n">
         <v>0</v>
@@ -2150,7 +2150,7 @@
         <v>0</v>
       </c>
       <c r="W15" t="n">
-        <v>0</v>
+        <v>-1.475462685247075</v>
       </c>
       <c r="X15" t="n">
         <v>0</v>
@@ -2159,19 +2159,19 @@
         <v>0</v>
       </c>
       <c r="Z15" t="n">
-        <v>0</v>
+        <v>-2.723285606951114</v>
       </c>
       <c r="AA15" t="n">
-        <v>0</v>
+        <v>1.576222444784207</v>
       </c>
       <c r="AB15" t="n">
-        <v>0</v>
+        <v>11.44831120197395</v>
       </c>
       <c r="AC15" t="n">
-        <v>0</v>
+        <v>13.67190820985699</v>
       </c>
       <c r="AD15" t="n">
-        <v>0</v>
+        <v>15.84842555965021</v>
       </c>
       <c r="AE15" t="n">
         <v>0</v>
@@ -2180,7 +2180,7 @@
         <v>0</v>
       </c>
       <c r="AG15" t="n">
-        <v>0</v>
+        <v>3.602246001538805</v>
       </c>
       <c r="AH15" t="n">
         <v>0</v>
@@ -2189,7 +2189,7 @@
         <v>0</v>
       </c>
       <c r="AJ15" t="n">
-        <v>0</v>
+        <v>5.530407213910946</v>
       </c>
       <c r="AK15" t="n">
         <v>0</v>
@@ -2198,21 +2198,21 @@
         <v>0</v>
       </c>
       <c r="AM15" t="n">
-        <v>0</v>
+        <v>5.139031126558099</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0</v>
+        <v>0.5454495722126946</v>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>5.049791993425586</v>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>18.74092126346848</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>38.39856510910838</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -2221,7 +2221,7 @@
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>1.124625794116042</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -2230,7 +2230,7 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>10.15530698853429</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -2239,19 +2239,19 @@
         <v>0</v>
       </c>
       <c r="M16" t="n">
-        <v>0</v>
+        <v>23.69877968611682</v>
       </c>
       <c r="N16" t="n">
-        <v>0</v>
+        <v>2.301202142182699</v>
       </c>
       <c r="O16" t="n">
-        <v>0</v>
+        <v>15.60550082657199</v>
       </c>
       <c r="P16" t="n">
-        <v>-17.95662139729773</v>
+        <v>25.36028734692464</v>
       </c>
       <c r="Q16" t="n">
-        <v>0</v>
+        <v>51.91216676124913</v>
       </c>
       <c r="R16" t="n">
         <v>0</v>
@@ -2260,7 +2260,7 @@
         <v>0</v>
       </c>
       <c r="T16" t="n">
-        <v>0</v>
+        <v>-1.475462685247074</v>
       </c>
       <c r="U16" t="n">
         <v>0</v>
@@ -2269,7 +2269,7 @@
         <v>0</v>
       </c>
       <c r="W16" t="n">
-        <v>0</v>
+        <v>-6.912828115024684</v>
       </c>
       <c r="X16" t="n">
         <v>0</v>
@@ -2278,19 +2278,19 @@
         <v>0</v>
       </c>
       <c r="Z16" t="n">
-        <v>0</v>
+        <v>-13.76609940898933</v>
       </c>
       <c r="AA16" t="n">
-        <v>0</v>
+        <v>3.508714021200267</v>
       </c>
       <c r="AB16" t="n">
-        <v>0</v>
+        <v>24.12121622154257</v>
       </c>
       <c r="AC16" t="n">
-        <v>0</v>
+        <v>38.5077583072274</v>
       </c>
       <c r="AD16" t="n">
-        <v>0</v>
+        <v>55.30620345657083</v>
       </c>
       <c r="AE16" t="n">
         <v>0</v>
@@ -2299,7 +2299,7 @@
         <v>0</v>
       </c>
       <c r="AG16" t="n">
-        <v>0</v>
+        <v>3.031657194942603</v>
       </c>
       <c r="AH16" t="n">
         <v>0</v>
@@ -2308,7 +2308,7 @@
         <v>0</v>
       </c>
       <c r="AJ16" t="n">
-        <v>0</v>
+        <v>7.76217934737705</v>
       </c>
       <c r="AK16" t="n">
         <v>0</v>
@@ -2317,21 +2317,21 @@
         <v>0</v>
       </c>
       <c r="AM16" t="n">
-        <v>0</v>
+        <v>6.456376566773256</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0</v>
+        <v>1.449521828263224</v>
       </c>
       <c r="B17" t="n">
-        <v>0</v>
+        <v>11.17828061640937</v>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>38.39856510910838</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>95.71472975852407</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
@@ -2340,7 +2340,7 @@
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>2.088945385966567</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -2349,7 +2349,7 @@
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>0</v>
+        <v>17.40650157142676</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
@@ -2358,19 +2358,19 @@
         <v>0</v>
       </c>
       <c r="M17" t="n">
-        <v>0</v>
+        <v>47.39092645945158</v>
       </c>
       <c r="N17" t="n">
-        <v>0</v>
+        <v>2.272781618054275</v>
       </c>
       <c r="O17" t="n">
-        <v>0</v>
+        <v>16.46798512610517</v>
       </c>
       <c r="P17" t="n">
-        <v>0</v>
+        <v>51.91216676124913</v>
       </c>
       <c r="Q17" t="n">
-        <v>-17.95662139729709</v>
+        <v>39.05462463097899</v>
       </c>
       <c r="R17" t="n">
         <v>0</v>
@@ -2379,7 +2379,7 @@
         <v>0</v>
       </c>
       <c r="T17" t="n">
-        <v>0</v>
+        <v>-2.723285606951114</v>
       </c>
       <c r="U17" t="n">
         <v>0</v>
@@ -2388,7 +2388,7 @@
         <v>0</v>
       </c>
       <c r="W17" t="n">
-        <v>0</v>
+        <v>-13.76609940898933</v>
       </c>
       <c r="X17" t="n">
         <v>0</v>
@@ -2397,19 +2397,19 @@
         <v>0</v>
       </c>
       <c r="Z17" t="n">
-        <v>0</v>
+        <v>-43.12718909070011</v>
       </c>
       <c r="AA17" t="n">
-        <v>0</v>
+        <v>4.512122142873354</v>
       </c>
       <c r="AB17" t="n">
-        <v>0</v>
+        <v>36.21567214747493</v>
       </c>
       <c r="AC17" t="n">
-        <v>0</v>
+        <v>78.68980267650088</v>
       </c>
       <c r="AD17" t="n">
-        <v>0</v>
+        <v>151.1499475879253</v>
       </c>
       <c r="AE17" t="n">
         <v>0</v>
@@ -2418,7 +2418,7 @@
         <v>0</v>
       </c>
       <c r="AG17" t="n">
-        <v>0</v>
+        <v>0.5487270400261994</v>
       </c>
       <c r="AH17" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
         <v>0</v>
       </c>
       <c r="AJ17" t="n">
-        <v>0</v>
+        <v>3.978407090882079</v>
       </c>
       <c r="AK17" t="n">
         <v>0</v>
@@ -2436,7 +2436,7 @@
         <v>0</v>
       </c>
       <c r="AM17" t="n">
-        <v>0</v>
+        <v>11.56233920550879</v>
       </c>
     </row>
     <row r="18">
@@ -2453,7 +2453,7 @@
         <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>0.01064078252761629</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
@@ -2462,7 +2462,7 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>0.3758371805596656</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
@@ -2471,7 +2471,7 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>0.8333571581880166</v>
       </c>
       <c r="L18" t="n">
         <v>0</v>
@@ -2492,7 +2492,7 @@
         <v>0</v>
       </c>
       <c r="R18" t="n">
-        <v>-9.507972103246219</v>
+        <v>1.192134315798659</v>
       </c>
       <c r="S18" t="n">
         <v>0</v>
@@ -2501,7 +2501,7 @@
         <v>0</v>
       </c>
       <c r="U18" t="n">
-        <v>0</v>
+        <v>1.766832501424194</v>
       </c>
       <c r="V18" t="n">
         <v>0</v>
@@ -2510,7 +2510,7 @@
         <v>0</v>
       </c>
       <c r="X18" t="n">
-        <v>0</v>
+        <v>1.382854560945209</v>
       </c>
       <c r="Y18" t="n">
         <v>0</v>
@@ -2531,7 +2531,7 @@
         <v>0</v>
       </c>
       <c r="AE18" t="n">
-        <v>0</v>
+        <v>0.7651230248262965</v>
       </c>
       <c r="AF18" t="n">
         <v>0</v>
@@ -2540,7 +2540,7 @@
         <v>0</v>
       </c>
       <c r="AH18" t="n">
-        <v>0</v>
+        <v>1.27280487236772</v>
       </c>
       <c r="AI18" t="n">
         <v>0</v>
@@ -2549,7 +2549,7 @@
         <v>0</v>
       </c>
       <c r="AK18" t="n">
-        <v>0</v>
+        <v>1.097514897426634</v>
       </c>
       <c r="AL18" t="n">
         <v>0</v>
@@ -2575,7 +2575,7 @@
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>0.01064078252761629</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
@@ -2584,7 +2584,7 @@
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>0.3758371805596658</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -2593,7 +2593,7 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>0</v>
+        <v>0.8333571581880166</v>
       </c>
       <c r="M19" t="n">
         <v>0</v>
@@ -2614,7 +2614,7 @@
         <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>-6.323852495613346</v>
+        <v>1.192134315798659</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -2623,7 +2623,7 @@
         <v>0</v>
       </c>
       <c r="V19" t="n">
-        <v>0</v>
+        <v>1.766832501424194</v>
       </c>
       <c r="W19" t="n">
         <v>0</v>
@@ -2632,7 +2632,7 @@
         <v>0</v>
       </c>
       <c r="Y19" t="n">
-        <v>0</v>
+        <v>1.382854560945209</v>
       </c>
       <c r="Z19" t="n">
         <v>0</v>
@@ -2653,7 +2653,7 @@
         <v>0</v>
       </c>
       <c r="AF19" t="n">
-        <v>0</v>
+        <v>0.7651230248262962</v>
       </c>
       <c r="AG19" t="n">
         <v>0</v>
@@ -2662,7 +2662,7 @@
         <v>0</v>
       </c>
       <c r="AI19" t="n">
-        <v>0</v>
+        <v>1.272804872367719</v>
       </c>
       <c r="AJ19" t="n">
         <v>0</v>
@@ -2671,7 +2671,7 @@
         <v>0</v>
       </c>
       <c r="AL19" t="n">
-        <v>0</v>
+        <v>1.097514897426633</v>
       </c>
       <c r="AM19" t="n">
         <v>0</v>
@@ -2679,16 +2679,16 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0</v>
+        <v>-0.004917756917705785</v>
       </c>
       <c r="B20" t="n">
-        <v>0</v>
+        <v>-0.1787429074991289</v>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>-1.124625794116042</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>-2.088945385966567</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -2697,7 +2697,7 @@
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>-0.2169371577703999</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
@@ -2706,7 +2706,7 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>-1.248713956425854</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
@@ -2715,19 +2715,19 @@
         <v>0</v>
       </c>
       <c r="M20" t="n">
-        <v>0</v>
+        <v>-0.9306538784753915</v>
       </c>
       <c r="N20" t="n">
-        <v>0</v>
+        <v>-0.03612803534483141</v>
       </c>
       <c r="O20" t="n">
-        <v>0</v>
+        <v>-0.5819261365744327</v>
       </c>
       <c r="P20" t="n">
-        <v>0</v>
+        <v>-1.475462685247074</v>
       </c>
       <c r="Q20" t="n">
-        <v>0</v>
+        <v>-2.723285606951114</v>
       </c>
       <c r="R20" t="n">
         <v>0</v>
@@ -2736,7 +2736,7 @@
         <v>0</v>
       </c>
       <c r="T20" t="n">
-        <v>-5.027470949428402</v>
+        <v>1.477838631755247</v>
       </c>
       <c r="U20" t="n">
         <v>0</v>
@@ -2745,7 +2745,7 @@
         <v>0</v>
       </c>
       <c r="W20" t="n">
-        <v>0</v>
+        <v>3.250101211246582</v>
       </c>
       <c r="X20" t="n">
         <v>0</v>
@@ -2754,19 +2754,19 @@
         <v>0</v>
       </c>
       <c r="Z20" t="n">
-        <v>0</v>
+        <v>3.194957394976628</v>
       </c>
       <c r="AA20" t="n">
-        <v>0</v>
+        <v>-0.6378678045689179</v>
       </c>
       <c r="AB20" t="n">
-        <v>0</v>
+        <v>-2.760336696370763</v>
       </c>
       <c r="AC20" t="n">
-        <v>0</v>
+        <v>-2.520531082126993</v>
       </c>
       <c r="AD20" t="n">
-        <v>0</v>
+        <v>-2.802640033063934</v>
       </c>
       <c r="AE20" t="n">
         <v>0</v>
@@ -2775,7 +2775,7 @@
         <v>0</v>
       </c>
       <c r="AG20" t="n">
-        <v>0</v>
+        <v>-0.2074482860328148</v>
       </c>
       <c r="AH20" t="n">
         <v>0</v>
@@ -2784,7 +2784,7 @@
         <v>0</v>
       </c>
       <c r="AJ20" t="n">
-        <v>0</v>
+        <v>0.8149003037378533</v>
       </c>
       <c r="AK20" t="n">
         <v>0</v>
@@ -2793,7 +2793,7 @@
         <v>0</v>
       </c>
       <c r="AM20" t="n">
-        <v>0</v>
+        <v>1.178655034612895</v>
       </c>
     </row>
     <row r="21">
@@ -2810,7 +2810,7 @@
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>0.3758371805596659</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
@@ -2819,7 +2819,7 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
+        <v>4.550080082221125</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
@@ -2828,7 +2828,7 @@
         <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>12.8982716519249</v>
       </c>
       <c r="L21" t="n">
         <v>0</v>
@@ -2849,7 +2849,7 @@
         <v>0</v>
       </c>
       <c r="R21" t="n">
-        <v>0</v>
+        <v>1.766832501424194</v>
       </c>
       <c r="S21" t="n">
         <v>0</v>
@@ -2858,7 +2858,7 @@
         <v>0</v>
       </c>
       <c r="U21" t="n">
-        <v>-4.77695853862113</v>
+        <v>-13.40329958962834</v>
       </c>
       <c r="V21" t="n">
         <v>0</v>
@@ -2867,7 +2867,7 @@
         <v>0</v>
       </c>
       <c r="X21" t="n">
-        <v>0</v>
+        <v>20.18728619194507</v>
       </c>
       <c r="Y21" t="n">
         <v>0</v>
@@ -2888,7 +2888,7 @@
         <v>0</v>
       </c>
       <c r="AE21" t="n">
-        <v>0</v>
+        <v>3.676068662738705</v>
       </c>
       <c r="AF21" t="n">
         <v>0</v>
@@ -2897,7 +2897,7 @@
         <v>0</v>
       </c>
       <c r="AH21" t="n">
-        <v>0</v>
+        <v>13.81389572988589</v>
       </c>
       <c r="AI21" t="n">
         <v>0</v>
@@ -2906,7 +2906,7 @@
         <v>0</v>
       </c>
       <c r="AK21" t="n">
-        <v>0</v>
+        <v>18.37925462552074</v>
       </c>
       <c r="AL21" t="n">
         <v>0</v>
@@ -2932,7 +2932,7 @@
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>0.3758371805596659</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
@@ -2941,7 +2941,7 @@
         <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>4.550080082221125</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -2950,7 +2950,7 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>0</v>
+        <v>12.8982716519249</v>
       </c>
       <c r="M22" t="n">
         <v>0</v>
@@ -2971,7 +2971,7 @@
         <v>0</v>
       </c>
       <c r="S22" t="n">
-        <v>0</v>
+        <v>1.766832501424194</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2980,7 +2980,7 @@
         <v>0</v>
       </c>
       <c r="V22" t="n">
-        <v>-4.776958538621041</v>
+        <v>-13.40329958962834</v>
       </c>
       <c r="W22" t="n">
         <v>0</v>
@@ -2989,7 +2989,7 @@
         <v>0</v>
       </c>
       <c r="Y22" t="n">
-        <v>0</v>
+        <v>20.18728619194507</v>
       </c>
       <c r="Z22" t="n">
         <v>0</v>
@@ -3010,7 +3010,7 @@
         <v>0</v>
       </c>
       <c r="AF22" t="n">
-        <v>0</v>
+        <v>3.676068662738704</v>
       </c>
       <c r="AG22" t="n">
         <v>0</v>
@@ -3019,7 +3019,7 @@
         <v>0</v>
       </c>
       <c r="AI22" t="n">
-        <v>0</v>
+        <v>13.81389572988588</v>
       </c>
       <c r="AJ22" t="n">
         <v>0</v>
@@ -3028,7 +3028,7 @@
         <v>0</v>
       </c>
       <c r="AL22" t="n">
-        <v>0</v>
+        <v>18.37925462552075</v>
       </c>
       <c r="AM22" t="n">
         <v>0</v>
@@ -3036,16 +3036,16 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>0</v>
+        <v>-0.4570860794626933</v>
       </c>
       <c r="B23" t="n">
-        <v>0</v>
+        <v>-3.971360158404172</v>
       </c>
       <c r="C23" t="n">
-        <v>0</v>
+        <v>-10.15530698853429</v>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>-17.40650157142676</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -3054,7 +3054,7 @@
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>-1.248713956425855</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
@@ -3063,7 +3063,7 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>-5.357830832620333</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
@@ -3072,19 +3072,19 @@
         <v>0</v>
       </c>
       <c r="M23" t="n">
-        <v>0</v>
+        <v>0.3636216678918154</v>
       </c>
       <c r="N23" t="n">
-        <v>0</v>
+        <v>-0.03074431601516749</v>
       </c>
       <c r="O23" t="n">
-        <v>0</v>
+        <v>-1.475462685247075</v>
       </c>
       <c r="P23" t="n">
-        <v>0</v>
+        <v>-6.912828115024684</v>
       </c>
       <c r="Q23" t="n">
-        <v>0</v>
+        <v>-13.76609940898933</v>
       </c>
       <c r="R23" t="n">
         <v>0</v>
@@ -3093,7 +3093,7 @@
         <v>0</v>
       </c>
       <c r="T23" t="n">
-        <v>0</v>
+        <v>3.250101211246582</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -3102,7 +3102,7 @@
         <v>0</v>
       </c>
       <c r="W23" t="n">
-        <v>0.5661697686769985</v>
+        <v>-7.381924980802701</v>
       </c>
       <c r="X23" t="n">
         <v>0</v>
@@ -3111,19 +3111,19 @@
         <v>0</v>
       </c>
       <c r="Z23" t="n">
-        <v>0</v>
+        <v>44.03641252598699</v>
       </c>
       <c r="AA23" t="n">
-        <v>0</v>
+        <v>-1.586326549568464</v>
       </c>
       <c r="AB23" t="n">
-        <v>0</v>
+        <v>-10.86627905110093</v>
       </c>
       <c r="AC23" t="n">
-        <v>0</v>
+        <v>-15.44425040665211</v>
       </c>
       <c r="AD23" t="n">
-        <v>0</v>
+        <v>-23.12502089407928</v>
       </c>
       <c r="AE23" t="n">
         <v>0</v>
@@ -3132,7 +3132,7 @@
         <v>0</v>
       </c>
       <c r="AG23" t="n">
-        <v>0</v>
+        <v>4.911791365184697</v>
       </c>
       <c r="AH23" t="n">
         <v>0</v>
@@ -3141,7 +3141,7 @@
         <v>0</v>
       </c>
       <c r="AJ23" t="n">
-        <v>0</v>
+        <v>16.06636222813914</v>
       </c>
       <c r="AK23" t="n">
         <v>0</v>
@@ -3150,7 +3150,7 @@
         <v>0</v>
       </c>
       <c r="AM23" t="n">
-        <v>0</v>
+        <v>28.31024971547307</v>
       </c>
     </row>
     <row r="24">
@@ -3167,7 +3167,7 @@
         <v>0</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>0.8333571581880173</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
@@ -3176,7 +3176,7 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>12.8982716519249</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
@@ -3185,7 +3185,7 @@
         <v>0</v>
       </c>
       <c r="K24" t="n">
-        <v>0</v>
+        <v>68.09819569804129</v>
       </c>
       <c r="L24" t="n">
         <v>0</v>
@@ -3206,7 +3206,7 @@
         <v>0</v>
       </c>
       <c r="R24" t="n">
-        <v>0</v>
+        <v>1.382854560945209</v>
       </c>
       <c r="S24" t="n">
         <v>0</v>
@@ -3215,7 +3215,7 @@
         <v>0</v>
       </c>
       <c r="U24" t="n">
-        <v>0</v>
+        <v>20.18728619194507</v>
       </c>
       <c r="V24" t="n">
         <v>0</v>
@@ -3224,7 +3224,7 @@
         <v>0</v>
       </c>
       <c r="X24" t="n">
-        <v>0.566169768677408</v>
+        <v>-486.8332616027242</v>
       </c>
       <c r="Y24" t="n">
         <v>0</v>
@@ -3245,7 +3245,7 @@
         <v>0</v>
       </c>
       <c r="AE24" t="n">
-        <v>0</v>
+        <v>4.518849650494094</v>
       </c>
       <c r="AF24" t="n">
         <v>0</v>
@@ -3254,7 +3254,7 @@
         <v>0</v>
       </c>
       <c r="AH24" t="n">
-        <v>0</v>
+        <v>37.24777675403165</v>
       </c>
       <c r="AI24" t="n">
         <v>0</v>
@@ -3263,7 +3263,7 @@
         <v>0</v>
       </c>
       <c r="AK24" t="n">
-        <v>0</v>
+        <v>129.7348004269145</v>
       </c>
       <c r="AL24" t="n">
         <v>0</v>
@@ -3289,7 +3289,7 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>0.8333571581880168</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
@@ -3298,7 +3298,7 @@
         <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
+        <v>12.89827165192491</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -3307,7 +3307,7 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>68.09819569804129</v>
       </c>
       <c r="M25" t="n">
         <v>0</v>
@@ -3328,7 +3328,7 @@
         <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>0</v>
+        <v>1.382854560945209</v>
       </c>
       <c r="T25" t="n">
         <v>0</v>
@@ -3337,7 +3337,7 @@
         <v>0</v>
       </c>
       <c r="V25" t="n">
-        <v>0</v>
+        <v>20.18728619194507</v>
       </c>
       <c r="W25" t="n">
         <v>0</v>
@@ -3346,7 +3346,7 @@
         <v>0</v>
       </c>
       <c r="Y25" t="n">
-        <v>0.6650602861264325</v>
+        <v>-486.8332616027242</v>
       </c>
       <c r="Z25" t="n">
         <v>0</v>
@@ -3367,7 +3367,7 @@
         <v>0</v>
       </c>
       <c r="AF25" t="n">
-        <v>0</v>
+        <v>4.518849650494094</v>
       </c>
       <c r="AG25" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
         <v>0</v>
       </c>
       <c r="AI25" t="n">
-        <v>0</v>
+        <v>37.24777675403165</v>
       </c>
       <c r="AJ25" t="n">
         <v>0</v>
@@ -3385,7 +3385,7 @@
         <v>0</v>
       </c>
       <c r="AL25" t="n">
-        <v>0</v>
+        <v>129.7348004269146</v>
       </c>
       <c r="AM25" t="n">
         <v>0</v>
@@ -3393,16 +3393,16 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>0</v>
+        <v>-1.16868944234641</v>
       </c>
       <c r="B26" t="n">
-        <v>0</v>
+        <v>-9.21881277318213</v>
       </c>
       <c r="C26" t="n">
-        <v>0</v>
+        <v>-23.69877968611681</v>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>-47.39092645945157</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
@@ -3411,7 +3411,7 @@
         <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>0</v>
+        <v>-0.930653878475391</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
@@ -3420,7 +3420,7 @@
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>0</v>
+        <v>0.3636216678918136</v>
       </c>
       <c r="K26" t="n">
         <v>0</v>
@@ -3429,19 +3429,19 @@
         <v>0</v>
       </c>
       <c r="M26" t="n">
-        <v>0</v>
+        <v>23.68879886756204</v>
       </c>
       <c r="N26" t="n">
-        <v>0</v>
+        <v>-0.03310305217715067</v>
       </c>
       <c r="O26" t="n">
-        <v>0</v>
+        <v>-2.723285606951114</v>
       </c>
       <c r="P26" t="n">
-        <v>0</v>
+        <v>-13.76609940898933</v>
       </c>
       <c r="Q26" t="n">
-        <v>0</v>
+        <v>-43.12718909070011</v>
       </c>
       <c r="R26" t="n">
         <v>0</v>
@@ -3450,7 +3450,7 @@
         <v>0</v>
       </c>
       <c r="T26" t="n">
-        <v>0</v>
+        <v>3.194957394976628</v>
       </c>
       <c r="U26" t="n">
         <v>0</v>
@@ -3459,7 +3459,7 @@
         <v>0</v>
       </c>
       <c r="W26" t="n">
-        <v>0</v>
+        <v>44.03641252598699</v>
       </c>
       <c r="X26" t="n">
         <v>0</v>
@@ -3468,19 +3468,19 @@
         <v>0</v>
       </c>
       <c r="Z26" t="n">
-        <v>0.9478815385520341</v>
+        <v>-436.8057222575121</v>
       </c>
       <c r="AA26" t="n">
-        <v>0</v>
+        <v>-1.877188462822925</v>
       </c>
       <c r="AB26" t="n">
-        <v>0</v>
+        <v>-17.2616970864677</v>
       </c>
       <c r="AC26" t="n">
-        <v>0</v>
+        <v>-34.62715650309303</v>
       </c>
       <c r="AD26" t="n">
-        <v>0</v>
+        <v>-60.6386162974352</v>
       </c>
       <c r="AE26" t="n">
         <v>0</v>
@@ -3489,7 +3489,7 @@
         <v>0</v>
       </c>
       <c r="AG26" t="n">
-        <v>0</v>
+        <v>8.709720073795213</v>
       </c>
       <c r="AH26" t="n">
         <v>0</v>
@@ -3498,7 +3498,7 @@
         <v>0</v>
       </c>
       <c r="AJ26" t="n">
-        <v>0</v>
+        <v>42.56472805406715</v>
       </c>
       <c r="AK26" t="n">
         <v>0</v>
@@ -3507,21 +3507,21 @@
         <v>0</v>
       </c>
       <c r="AM26" t="n">
-        <v>0</v>
+        <v>145.0244454550882</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>0</v>
+        <v>0.05955589180169553</v>
       </c>
       <c r="B27" t="n">
-        <v>0</v>
+        <v>1.576222444784207</v>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>3.508714021200267</v>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>4.512122142873354</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
@@ -3530,7 +3530,7 @@
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>0</v>
+        <v>0.6378678045689179</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
@@ -3539,7 +3539,7 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
+        <v>1.586326549568464</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
@@ -3548,19 +3548,19 @@
         <v>0</v>
       </c>
       <c r="M27" t="n">
-        <v>0</v>
+        <v>1.877188462822925</v>
       </c>
       <c r="N27" t="n">
-        <v>0</v>
+        <v>0.05955589180169553</v>
       </c>
       <c r="O27" t="n">
-        <v>0</v>
+        <v>1.576222444784207</v>
       </c>
       <c r="P27" t="n">
-        <v>0</v>
+        <v>3.508714021200267</v>
       </c>
       <c r="Q27" t="n">
-        <v>0</v>
+        <v>4.512122142873354</v>
       </c>
       <c r="R27" t="n">
         <v>0</v>
@@ -3569,7 +3569,7 @@
         <v>0</v>
       </c>
       <c r="T27" t="n">
-        <v>0</v>
+        <v>-0.6378678045689179</v>
       </c>
       <c r="U27" t="n">
         <v>0</v>
@@ -3578,7 +3578,7 @@
         <v>0</v>
       </c>
       <c r="W27" t="n">
-        <v>0</v>
+        <v>-1.586326549568464</v>
       </c>
       <c r="X27" t="n">
         <v>0</v>
@@ -3587,19 +3587,19 @@
         <v>0</v>
       </c>
       <c r="Z27" t="n">
-        <v>0</v>
+        <v>-1.877188462822925</v>
       </c>
       <c r="AA27" t="n">
-        <v>1.284165238006862</v>
+        <v>7.31231103509213</v>
       </c>
       <c r="AB27" t="n">
-        <v>0</v>
+        <v>9.566067929219599</v>
       </c>
       <c r="AC27" t="n">
-        <v>0</v>
+        <v>5.02662268669918</v>
       </c>
       <c r="AD27" t="n">
-        <v>0</v>
+        <v>5.060475449234733</v>
       </c>
       <c r="AE27" t="n">
         <v>0</v>
@@ -3631,16 +3631,16 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>0</v>
+        <v>1.418553104775894</v>
       </c>
       <c r="B28" t="n">
-        <v>0</v>
+        <v>11.44831120197395</v>
       </c>
       <c r="C28" t="n">
-        <v>0</v>
+        <v>24.12121622154257</v>
       </c>
       <c r="D28" t="n">
-        <v>0</v>
+        <v>36.21567214747493</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
@@ -3649,7 +3649,7 @@
         <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>0</v>
+        <v>2.760336696370763</v>
       </c>
       <c r="H28" t="n">
         <v>0</v>
@@ -3658,7 +3658,7 @@
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>0</v>
+        <v>10.86627905110093</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
@@ -3667,19 +3667,19 @@
         <v>0</v>
       </c>
       <c r="M28" t="n">
-        <v>0</v>
+        <v>17.2616970864677</v>
       </c>
       <c r="N28" t="n">
-        <v>0</v>
+        <v>1.418553104775894</v>
       </c>
       <c r="O28" t="n">
-        <v>0</v>
+        <v>11.44831120197395</v>
       </c>
       <c r="P28" t="n">
-        <v>0</v>
+        <v>24.12121622154257</v>
       </c>
       <c r="Q28" t="n">
-        <v>0</v>
+        <v>36.21567214747493</v>
       </c>
       <c r="R28" t="n">
         <v>0</v>
@@ -3688,7 +3688,7 @@
         <v>0</v>
       </c>
       <c r="T28" t="n">
-        <v>0</v>
+        <v>-2.760336696370763</v>
       </c>
       <c r="U28" t="n">
         <v>0</v>
@@ -3697,7 +3697,7 @@
         <v>0</v>
       </c>
       <c r="W28" t="n">
-        <v>0</v>
+        <v>-10.86627905110093</v>
       </c>
       <c r="X28" t="n">
         <v>0</v>
@@ -3706,19 +3706,19 @@
         <v>0</v>
       </c>
       <c r="Z28" t="n">
-        <v>0</v>
+        <v>-17.2616970864677</v>
       </c>
       <c r="AA28" t="n">
-        <v>0</v>
+        <v>9.566067929219599</v>
       </c>
       <c r="AB28" t="n">
-        <v>1.284165238006926</v>
+        <v>33.85330624567014</v>
       </c>
       <c r="AC28" t="n">
-        <v>0</v>
+        <v>36.22964287190445</v>
       </c>
       <c r="AD28" t="n">
-        <v>0</v>
+        <v>41.72869520649253</v>
       </c>
       <c r="AE28" t="n">
         <v>0</v>
@@ -3750,16 +3750,16 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>0</v>
+        <v>1.831416724125386</v>
       </c>
       <c r="B29" t="n">
-        <v>0</v>
+        <v>13.67190820985699</v>
       </c>
       <c r="C29" t="n">
-        <v>0</v>
+        <v>38.5077583072274</v>
       </c>
       <c r="D29" t="n">
-        <v>0</v>
+        <v>78.68980267650088</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
@@ -3768,7 +3768,7 @@
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>0</v>
+        <v>2.520531082126993</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
@@ -3777,7 +3777,7 @@
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>0</v>
+        <v>15.44425040665211</v>
       </c>
       <c r="K29" t="n">
         <v>0</v>
@@ -3786,19 +3786,19 @@
         <v>0</v>
       </c>
       <c r="M29" t="n">
-        <v>0</v>
+        <v>34.62715650309303</v>
       </c>
       <c r="N29" t="n">
-        <v>0</v>
+        <v>1.831416724125386</v>
       </c>
       <c r="O29" t="n">
-        <v>0</v>
+        <v>13.67190820985699</v>
       </c>
       <c r="P29" t="n">
-        <v>0</v>
+        <v>38.5077583072274</v>
       </c>
       <c r="Q29" t="n">
-        <v>0</v>
+        <v>78.68980267650088</v>
       </c>
       <c r="R29" t="n">
         <v>0</v>
@@ -3807,7 +3807,7 @@
         <v>0</v>
       </c>
       <c r="T29" t="n">
-        <v>0</v>
+        <v>-2.520531082126993</v>
       </c>
       <c r="U29" t="n">
         <v>0</v>
@@ -3816,7 +3816,7 @@
         <v>0</v>
       </c>
       <c r="W29" t="n">
-        <v>0</v>
+        <v>-15.44425040665211</v>
       </c>
       <c r="X29" t="n">
         <v>0</v>
@@ -3825,19 +3825,19 @@
         <v>0</v>
       </c>
       <c r="Z29" t="n">
-        <v>0</v>
+        <v>-34.62715650309303</v>
       </c>
       <c r="AA29" t="n">
-        <v>0</v>
+        <v>5.02662268669918</v>
       </c>
       <c r="AB29" t="n">
-        <v>0</v>
+        <v>36.22964287190445</v>
       </c>
       <c r="AC29" t="n">
-        <v>1.541161854938243</v>
+        <v>38.28138756538412</v>
       </c>
       <c r="AD29" t="n">
-        <v>0</v>
+        <v>94.62701925298215</v>
       </c>
       <c r="AE29" t="n">
         <v>0</v>
@@ -3869,16 +3869,16 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>0</v>
+        <v>2.138875613550525</v>
       </c>
       <c r="B30" t="n">
-        <v>0</v>
+        <v>15.84842555965021</v>
       </c>
       <c r="C30" t="n">
-        <v>0</v>
+        <v>55.30620345657083</v>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>151.1499475879253</v>
       </c>
       <c r="E30" t="n">
         <v>0</v>
@@ -3887,7 +3887,7 @@
         <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>0</v>
+        <v>2.802640033063934</v>
       </c>
       <c r="H30" t="n">
         <v>0</v>
@@ -3896,7 +3896,7 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>0</v>
+        <v>23.12502089407928</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
@@ -3905,19 +3905,19 @@
         <v>0</v>
       </c>
       <c r="M30" t="n">
-        <v>0</v>
+        <v>60.6386162974352</v>
       </c>
       <c r="N30" t="n">
-        <v>0</v>
+        <v>2.138875613550525</v>
       </c>
       <c r="O30" t="n">
-        <v>0</v>
+        <v>15.84842555965021</v>
       </c>
       <c r="P30" t="n">
-        <v>0</v>
+        <v>55.30620345657083</v>
       </c>
       <c r="Q30" t="n">
-        <v>0</v>
+        <v>151.1499475879253</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -3926,7 +3926,7 @@
         <v>0</v>
       </c>
       <c r="T30" t="n">
-        <v>0</v>
+        <v>-2.802640033063934</v>
       </c>
       <c r="U30" t="n">
         <v>0</v>
@@ -3935,7 +3935,7 @@
         <v>0</v>
       </c>
       <c r="W30" t="n">
-        <v>0</v>
+        <v>-23.12502089407928</v>
       </c>
       <c r="X30" t="n">
         <v>0</v>
@@ -3944,19 +3944,19 @@
         <v>0</v>
       </c>
       <c r="Z30" t="n">
-        <v>0</v>
+        <v>-60.6386162974352</v>
       </c>
       <c r="AA30" t="n">
-        <v>0</v>
+        <v>5.060475449234733</v>
       </c>
       <c r="AB30" t="n">
-        <v>0</v>
+        <v>41.72869520649253</v>
       </c>
       <c r="AC30" t="n">
-        <v>0</v>
+        <v>94.62701925298215</v>
       </c>
       <c r="AD30" t="n">
-        <v>2.724611937281866</v>
+        <v>1.784547761482713</v>
       </c>
       <c r="AE30" t="n">
         <v>0</v>
@@ -4000,7 +4000,7 @@
         <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>0</v>
+        <v>0.7651230248262965</v>
       </c>
       <c r="F31" t="n">
         <v>0</v>
@@ -4009,7 +4009,7 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>3.676068662738705</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>
@@ -4018,7 +4018,7 @@
         <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>0</v>
+        <v>4.518849650494094</v>
       </c>
       <c r="L31" t="n">
         <v>0</v>
@@ -4039,7 +4039,7 @@
         <v>0</v>
       </c>
       <c r="R31" t="n">
-        <v>0</v>
+        <v>0.7651230248262965</v>
       </c>
       <c r="S31" t="n">
         <v>0</v>
@@ -4048,7 +4048,7 @@
         <v>0</v>
       </c>
       <c r="U31" t="n">
-        <v>0</v>
+        <v>3.676068662738705</v>
       </c>
       <c r="V31" t="n">
         <v>0</v>
@@ -4057,7 +4057,7 @@
         <v>0</v>
       </c>
       <c r="X31" t="n">
-        <v>0</v>
+        <v>4.518849650494094</v>
       </c>
       <c r="Y31" t="n">
         <v>0</v>
@@ -4078,7 +4078,7 @@
         <v>0</v>
       </c>
       <c r="AE31" t="n">
-        <v>3.249959986581969</v>
+        <v>1.73621494614338</v>
       </c>
       <c r="AF31" t="n">
         <v>0</v>
@@ -4087,7 +4087,7 @@
         <v>0</v>
       </c>
       <c r="AH31" t="n">
-        <v>0</v>
+        <v>5.17361296662818</v>
       </c>
       <c r="AI31" t="n">
         <v>0</v>
@@ -4096,7 +4096,7 @@
         <v>0</v>
       </c>
       <c r="AK31" t="n">
-        <v>0</v>
+        <v>4.519611486538499</v>
       </c>
       <c r="AL31" t="n">
         <v>0</v>
@@ -4122,7 +4122,7 @@
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>0.7651230248262962</v>
       </c>
       <c r="G32" t="n">
         <v>0</v>
@@ -4131,7 +4131,7 @@
         <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>3.676068662738704</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -4140,7 +4140,7 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>0</v>
+        <v>4.518849650494094</v>
       </c>
       <c r="M32" t="n">
         <v>0</v>
@@ -4161,7 +4161,7 @@
         <v>0</v>
       </c>
       <c r="S32" t="n">
-        <v>0</v>
+        <v>0.7651230248262962</v>
       </c>
       <c r="T32" t="n">
         <v>0</v>
@@ -4170,7 +4170,7 @@
         <v>0</v>
       </c>
       <c r="V32" t="n">
-        <v>0</v>
+        <v>3.676068662738704</v>
       </c>
       <c r="W32" t="n">
         <v>0</v>
@@ -4179,7 +4179,7 @@
         <v>0</v>
       </c>
       <c r="Y32" t="n">
-        <v>0</v>
+        <v>4.518849650494094</v>
       </c>
       <c r="Z32" t="n">
         <v>0</v>
@@ -4200,7 +4200,7 @@
         <v>0</v>
       </c>
       <c r="AF32" t="n">
-        <v>3.664462994468991</v>
+        <v>1.73621494614338</v>
       </c>
       <c r="AG32" t="n">
         <v>0</v>
@@ -4209,7 +4209,7 @@
         <v>0</v>
       </c>
       <c r="AI32" t="n">
-        <v>0</v>
+        <v>5.17361296662818</v>
       </c>
       <c r="AJ32" t="n">
         <v>0</v>
@@ -4218,7 +4218,7 @@
         <v>0</v>
       </c>
       <c r="AL32" t="n">
-        <v>0</v>
+        <v>4.519611486538499</v>
       </c>
       <c r="AM32" t="n">
         <v>0</v>
@@ -4226,16 +4226,16 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>0</v>
+        <v>-0.5964506393073215</v>
       </c>
       <c r="B33" t="n">
-        <v>0</v>
+        <v>-3.602246001538805</v>
       </c>
       <c r="C33" t="n">
-        <v>0</v>
+        <v>-3.031657194942603</v>
       </c>
       <c r="D33" t="n">
-        <v>0</v>
+        <v>-0.5487270400261994</v>
       </c>
       <c r="E33" t="n">
         <v>0</v>
@@ -4244,7 +4244,7 @@
         <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>0</v>
+        <v>-0.2074482860328148</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
@@ -4253,7 +4253,7 @@
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>0</v>
+        <v>4.911791365184697</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
@@ -4262,19 +4262,19 @@
         <v>0</v>
       </c>
       <c r="M33" t="n">
-        <v>0</v>
+        <v>8.709720073795213</v>
       </c>
       <c r="N33" t="n">
-        <v>0</v>
+        <v>0.5964506393073215</v>
       </c>
       <c r="O33" t="n">
-        <v>0</v>
+        <v>3.602246001538805</v>
       </c>
       <c r="P33" t="n">
-        <v>0</v>
+        <v>3.031657194942603</v>
       </c>
       <c r="Q33" t="n">
-        <v>0</v>
+        <v>0.5487270400261994</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -4283,7 +4283,7 @@
         <v>0</v>
       </c>
       <c r="T33" t="n">
-        <v>0</v>
+        <v>-0.2074482860328148</v>
       </c>
       <c r="U33" t="n">
         <v>0</v>
@@ -4292,7 +4292,7 @@
         <v>0</v>
       </c>
       <c r="W33" t="n">
-        <v>0</v>
+        <v>4.911791365184697</v>
       </c>
       <c r="X33" t="n">
         <v>0</v>
@@ -4301,7 +4301,7 @@
         <v>0</v>
       </c>
       <c r="Z33" t="n">
-        <v>0</v>
+        <v>8.709720073795213</v>
       </c>
       <c r="AA33" t="n">
         <v>0</v>
@@ -4322,7 +4322,7 @@
         <v>0</v>
       </c>
       <c r="AG33" t="n">
-        <v>11.16549252035082</v>
+        <v>5.38670493979505</v>
       </c>
       <c r="AH33" t="n">
         <v>0</v>
@@ -4331,7 +4331,7 @@
         <v>0</v>
       </c>
       <c r="AJ33" t="n">
-        <v>0</v>
+        <v>10.35444592154595</v>
       </c>
       <c r="AK33" t="n">
         <v>0</v>
@@ -4340,7 +4340,7 @@
         <v>0</v>
       </c>
       <c r="AM33" t="n">
-        <v>0</v>
+        <v>10.81502174551066</v>
       </c>
     </row>
     <row r="34">
@@ -4357,7 +4357,7 @@
         <v>0</v>
       </c>
       <c r="E34" t="n">
-        <v>0</v>
+        <v>1.27280487236772</v>
       </c>
       <c r="F34" t="n">
         <v>0</v>
@@ -4366,7 +4366,7 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>13.81389572988589</v>
       </c>
       <c r="I34" t="n">
         <v>0</v>
@@ -4375,7 +4375,7 @@
         <v>0</v>
       </c>
       <c r="K34" t="n">
-        <v>0</v>
+        <v>37.24777675403165</v>
       </c>
       <c r="L34" t="n">
         <v>0</v>
@@ -4396,7 +4396,7 @@
         <v>0</v>
       </c>
       <c r="R34" t="n">
-        <v>0</v>
+        <v>1.27280487236772</v>
       </c>
       <c r="S34" t="n">
         <v>0</v>
@@ -4405,7 +4405,7 @@
         <v>0</v>
       </c>
       <c r="U34" t="n">
-        <v>0</v>
+        <v>13.81389572988589</v>
       </c>
       <c r="V34" t="n">
         <v>0</v>
@@ -4414,7 +4414,7 @@
         <v>0</v>
       </c>
       <c r="X34" t="n">
-        <v>0</v>
+        <v>37.24777675403165</v>
       </c>
       <c r="Y34" t="n">
         <v>0</v>
@@ -4435,7 +4435,7 @@
         <v>0</v>
       </c>
       <c r="AE34" t="n">
-        <v>0</v>
+        <v>5.17361296662818</v>
       </c>
       <c r="AF34" t="n">
         <v>0</v>
@@ -4444,7 +4444,7 @@
         <v>0</v>
       </c>
       <c r="AH34" t="n">
-        <v>11.27769499484176</v>
+        <v>-65.91517041382774</v>
       </c>
       <c r="AI34" t="n">
         <v>0</v>
@@ -4453,7 +4453,7 @@
         <v>0</v>
       </c>
       <c r="AK34" t="n">
-        <v>0</v>
+        <v>47.8711030872023</v>
       </c>
       <c r="AL34" t="n">
         <v>0</v>
@@ -4479,7 +4479,7 @@
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>0</v>
+        <v>1.272804872367719</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
@@ -4488,7 +4488,7 @@
         <v>0</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
+        <v>13.81389572988588</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -4497,7 +4497,7 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>0</v>
+        <v>37.24777675403165</v>
       </c>
       <c r="M35" t="n">
         <v>0</v>
@@ -4518,7 +4518,7 @@
         <v>0</v>
       </c>
       <c r="S35" t="n">
-        <v>0</v>
+        <v>1.272804872367719</v>
       </c>
       <c r="T35" t="n">
         <v>0</v>
@@ -4527,7 +4527,7 @@
         <v>0</v>
       </c>
       <c r="V35" t="n">
-        <v>0</v>
+        <v>13.81389572988588</v>
       </c>
       <c r="W35" t="n">
         <v>0</v>
@@ -4536,7 +4536,7 @@
         <v>0</v>
       </c>
       <c r="Y35" t="n">
-        <v>0</v>
+        <v>37.24777675403165</v>
       </c>
       <c r="Z35" t="n">
         <v>0</v>
@@ -4557,7 +4557,7 @@
         <v>0</v>
       </c>
       <c r="AF35" t="n">
-        <v>0</v>
+        <v>5.17361296662818</v>
       </c>
       <c r="AG35" t="n">
         <v>0</v>
@@ -4566,7 +4566,7 @@
         <v>0</v>
       </c>
       <c r="AI35" t="n">
-        <v>11.6579762866647</v>
+        <v>-65.91517041382774</v>
       </c>
       <c r="AJ35" t="n">
         <v>0</v>
@@ -4575,7 +4575,7 @@
         <v>0</v>
       </c>
       <c r="AL35" t="n">
-        <v>0</v>
+        <v>47.87110308720229</v>
       </c>
       <c r="AM35" t="n">
         <v>0</v>
@@ -4583,16 +4583,16 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>0</v>
+        <v>-0.773537103112676</v>
       </c>
       <c r="B36" t="n">
-        <v>0</v>
+        <v>-5.530407213910946</v>
       </c>
       <c r="C36" t="n">
-        <v>0</v>
+        <v>-7.76217934737705</v>
       </c>
       <c r="D36" t="n">
-        <v>0</v>
+        <v>-3.978407090882079</v>
       </c>
       <c r="E36" t="n">
         <v>0</v>
@@ -4601,7 +4601,7 @@
         <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>0</v>
+        <v>0.8149003037378533</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
@@ -4610,7 +4610,7 @@
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
+        <v>16.06636222813914</v>
       </c>
       <c r="K36" t="n">
         <v>0</v>
@@ -4619,19 +4619,19 @@
         <v>0</v>
       </c>
       <c r="M36" t="n">
-        <v>0</v>
+        <v>42.56472805406715</v>
       </c>
       <c r="N36" t="n">
-        <v>0</v>
+        <v>0.773537103112676</v>
       </c>
       <c r="O36" t="n">
-        <v>0</v>
+        <v>5.530407213910946</v>
       </c>
       <c r="P36" t="n">
-        <v>0</v>
+        <v>7.76217934737705</v>
       </c>
       <c r="Q36" t="n">
-        <v>0</v>
+        <v>3.978407090882079</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -4640,7 +4640,7 @@
         <v>0</v>
       </c>
       <c r="T36" t="n">
-        <v>0</v>
+        <v>0.8149003037378533</v>
       </c>
       <c r="U36" t="n">
         <v>0</v>
@@ -4649,7 +4649,7 @@
         <v>0</v>
       </c>
       <c r="W36" t="n">
-        <v>0</v>
+        <v>16.06636222813914</v>
       </c>
       <c r="X36" t="n">
         <v>0</v>
@@ -4658,7 +4658,7 @@
         <v>0</v>
       </c>
       <c r="Z36" t="n">
-        <v>0</v>
+        <v>42.56472805406715</v>
       </c>
       <c r="AA36" t="n">
         <v>0</v>
@@ -4679,7 +4679,7 @@
         <v>0</v>
       </c>
       <c r="AG36" t="n">
-        <v>0</v>
+        <v>10.35444592154595</v>
       </c>
       <c r="AH36" t="n">
         <v>0</v>
@@ -4688,7 +4688,7 @@
         <v>0</v>
       </c>
       <c r="AJ36" t="n">
-        <v>11.65797628666481</v>
+        <v>-55.89272985088042</v>
       </c>
       <c r="AK36" t="n">
         <v>0</v>
@@ -4697,7 +4697,7 @@
         <v>0</v>
       </c>
       <c r="AM36" t="n">
-        <v>0</v>
+        <v>63.78466195801781</v>
       </c>
     </row>
     <row r="37">
@@ -4714,7 +4714,7 @@
         <v>0</v>
       </c>
       <c r="E37" t="n">
-        <v>0</v>
+        <v>1.097514897426634</v>
       </c>
       <c r="F37" t="n">
         <v>0</v>
@@ -4723,7 +4723,7 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>18.37925462552074</v>
       </c>
       <c r="I37" t="n">
         <v>0</v>
@@ -4732,7 +4732,7 @@
         <v>0</v>
       </c>
       <c r="K37" t="n">
-        <v>0</v>
+        <v>129.7348004269145</v>
       </c>
       <c r="L37" t="n">
         <v>0</v>
@@ -4753,7 +4753,7 @@
         <v>0</v>
       </c>
       <c r="R37" t="n">
-        <v>0</v>
+        <v>1.097514897426634</v>
       </c>
       <c r="S37" t="n">
         <v>0</v>
@@ -4762,7 +4762,7 @@
         <v>0</v>
       </c>
       <c r="U37" t="n">
-        <v>0</v>
+        <v>18.37925462552074</v>
       </c>
       <c r="V37" t="n">
         <v>0</v>
@@ -4771,7 +4771,7 @@
         <v>0</v>
       </c>
       <c r="X37" t="n">
-        <v>0</v>
+        <v>129.7348004269145</v>
       </c>
       <c r="Y37" t="n">
         <v>0</v>
@@ -4792,7 +4792,7 @@
         <v>0</v>
       </c>
       <c r="AE37" t="n">
-        <v>0</v>
+        <v>4.519611486538499</v>
       </c>
       <c r="AF37" t="n">
         <v>0</v>
@@ -4801,7 +4801,7 @@
         <v>0</v>
       </c>
       <c r="AH37" t="n">
-        <v>0</v>
+        <v>47.8711030872023</v>
       </c>
       <c r="AI37" t="n">
         <v>0</v>
@@ -4810,7 +4810,7 @@
         <v>0</v>
       </c>
       <c r="AK37" t="n">
-        <v>27.34326986756605</v>
+        <v>-2793.434313004652</v>
       </c>
       <c r="AL37" t="n">
         <v>0</v>
@@ -4836,7 +4836,7 @@
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>0</v>
+        <v>1.097514897426633</v>
       </c>
       <c r="G38" t="n">
         <v>0</v>
@@ -4845,7 +4845,7 @@
         <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>18.37925462552075</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -4854,7 +4854,7 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>0</v>
+        <v>129.7348004269146</v>
       </c>
       <c r="M38" t="n">
         <v>0</v>
@@ -4875,7 +4875,7 @@
         <v>0</v>
       </c>
       <c r="S38" t="n">
-        <v>0</v>
+        <v>1.097514897426633</v>
       </c>
       <c r="T38" t="n">
         <v>0</v>
@@ -4884,7 +4884,7 @@
         <v>0</v>
       </c>
       <c r="V38" t="n">
-        <v>0</v>
+        <v>18.37925462552075</v>
       </c>
       <c r="W38" t="n">
         <v>0</v>
@@ -4893,7 +4893,7 @@
         <v>0</v>
       </c>
       <c r="Y38" t="n">
-        <v>0</v>
+        <v>129.7348004269146</v>
       </c>
       <c r="Z38" t="n">
         <v>0</v>
@@ -4914,7 +4914,7 @@
         <v>0</v>
       </c>
       <c r="AF38" t="n">
-        <v>0</v>
+        <v>4.519611486538499</v>
       </c>
       <c r="AG38" t="n">
         <v>0</v>
@@ -4923,7 +4923,7 @@
         <v>0</v>
       </c>
       <c r="AI38" t="n">
-        <v>0</v>
+        <v>47.87110308720229</v>
       </c>
       <c r="AJ38" t="n">
         <v>0</v>
@@ -4932,7 +4932,7 @@
         <v>0</v>
       </c>
       <c r="AL38" t="n">
-        <v>40.05967303184045</v>
+        <v>-2793.434313004652</v>
       </c>
       <c r="AM38" t="n">
         <v>0</v>
@@ -4940,16 +4940,16 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>0</v>
+        <v>-0.8272631971284673</v>
       </c>
       <c r="B39" t="n">
-        <v>0</v>
+        <v>-5.139031126558099</v>
       </c>
       <c r="C39" t="n">
-        <v>0</v>
+        <v>-6.456376566773256</v>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>-11.56233920550879</v>
       </c>
       <c r="E39" t="n">
         <v>0</v>
@@ -4958,7 +4958,7 @@
         <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>0</v>
+        <v>1.178655034612895</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
@@ -4967,7 +4967,7 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>0</v>
+        <v>28.31024971547307</v>
       </c>
       <c r="K39" t="n">
         <v>0</v>
@@ -4976,19 +4976,19 @@
         <v>0</v>
       </c>
       <c r="M39" t="n">
-        <v>0</v>
+        <v>145.0244454550882</v>
       </c>
       <c r="N39" t="n">
-        <v>0</v>
+        <v>0.8272631971284673</v>
       </c>
       <c r="O39" t="n">
-        <v>0</v>
+        <v>5.139031126558099</v>
       </c>
       <c r="P39" t="n">
-        <v>0</v>
+        <v>6.456376566773256</v>
       </c>
       <c r="Q39" t="n">
-        <v>0</v>
+        <v>11.56233920550879</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -4997,7 +4997,7 @@
         <v>0</v>
       </c>
       <c r="T39" t="n">
-        <v>0</v>
+        <v>1.178655034612895</v>
       </c>
       <c r="U39" t="n">
         <v>0</v>
@@ -5006,7 +5006,7 @@
         <v>0</v>
       </c>
       <c r="W39" t="n">
-        <v>0</v>
+        <v>28.31024971547307</v>
       </c>
       <c r="X39" t="n">
         <v>0</v>
@@ -5015,7 +5015,7 @@
         <v>0</v>
       </c>
       <c r="Z39" t="n">
-        <v>0</v>
+        <v>145.0244454550882</v>
       </c>
       <c r="AA39" t="n">
         <v>0</v>
@@ -5036,7 +5036,7 @@
         <v>0</v>
       </c>
       <c r="AG39" t="n">
-        <v>0</v>
+        <v>10.81502174551066</v>
       </c>
       <c r="AH39" t="n">
         <v>0</v>
@@ -5045,7 +5045,7 @@
         <v>0</v>
       </c>
       <c r="AJ39" t="n">
-        <v>0</v>
+        <v>63.78466195801781</v>
       </c>
       <c r="AK39" t="n">
         <v>0</v>
@@ -5054,7 +5054,7 @@
         <v>0</v>
       </c>
       <c r="AM39" t="n">
-        <v>459.1634949960236</v>
+        <v>-2754.828586295333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>